<commit_message>
Structure exports keep a tension member's bending
A tension member with bending = true is written as a frame (IFC4
analysis view RIGID_JOINED_MEMBER, SAF Standard) with its tension-only
behaviour as information: OHL_Member Kind tension and Bending true, the
analysis member's Description, SAF Layer, CSV bending column. Members
with check = false are exported as any other, flagged (Check false,
"not checked", CSV check column). The every-profile sample gains one of
each; samples regenerated, IfcOpenShell checks: 12 files, 0 errors.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/exports/every-profile-saf.xlsx
+++ b/examples/exports/every-profile-saf.xlsx
@@ -2013,9 +2013,14 @@
       <c r="W6">
         <v>0</v>
       </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OHL: tension only, bending</t>
+        </is>
+      </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Axial force only</t>
+          <t xml:space="preserve">Standard</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -2328,6 +2333,11 @@
       </c>
       <c r="W10">
         <v>0</v>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OHL: not checked</t>
+        </is>
       </c>
       <c r="Y10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Structure types: no point on a member, a joint inserted; the link follows edits
A point needs a joint (owner decision 2026-10-21). Files that place one
along a member (member + at) are read with an attach joint inserted there
and the member split into continuous pieces (same fields, each buckling
over the whole member); the structure file as edited is written so, and
OHL-Structure's edits gain insert_joint. The FE share to the member ends
and the analysis-only split are removed; a joint only bars meet, loaded
across them, is refused with the fix. every-profile written on its joint:
the same numbers as before (frame).

In a structure file a point on a joint moved stays on it, its offset
recomputed (the joint no longer moves); only attach joints take a link.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/exports/every-profile-saf.xlsx
+++ b/examples/exports/every-profile-saf.xlsx
@@ -314,12 +314,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">On beam</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">m-EA</t>
+          <t xml:space="preserve">In node</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
         </is>
       </c>
       <c r="G2">
@@ -334,22 +334,6 @@
         <is>
           <t xml:space="preserve">Global</t>
         </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">From start</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Relative</t>
-        </is>
-      </c>
-      <c r="M2">
-        <v>0.25</v>
-      </c>
-      <c r="N2">
-        <v>1</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -1480,6 +1464,27 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1</t>
+        </is>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>1.25</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2e8efe3f-045f-c74d-fa98-07824f8fefe3</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -1647,7 +1652,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N0; N1</t>
+          <t xml:space="preserve">N0; P1</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1656,7 +1661,7 @@
         </is>
       </c>
       <c r="H2">
-        <v>5</v>
+        <v>1.25</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -2347,6 +2352,85 @@
       <c r="AB10" t="inlineStr">
         <is>
           <t xml:space="preserve">d1accef0-e745-bb7f-f3bd-621fa49762b1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">m-EA-2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">General</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EA-61x7</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P1; N1</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Line</t>
+        </is>
+      </c>
+      <c r="H11">
+        <v>3.75</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Line</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">z by vector</t>
+        </is>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <v>1</v>
+      </c>
+      <c r="N11">
+        <v>0</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Centre</t>
+        </is>
+      </c>
+      <c r="T11">
+        <v>0</v>
+      </c>
+      <c r="U11">
+        <v>0</v>
+      </c>
+      <c r="V11">
+        <v>0</v>
+      </c>
+      <c r="W11">
+        <v>0</v>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6aec4d59-2297-a85d-340e-0b9408de3fce</t>
         </is>
       </c>
     </row>

</xml_diff>